<commit_message>
fix: align demo source paths with employee workspace upload root
</commit_message>
<xml_diff>
--- a/capabilities/waste-specialist/examples/模拟制造企业-202608-09.xlsx
+++ b/capabilities/waste-specialist/examples/模拟制造企业-202608-09.xlsx
@@ -536,13 +536,6 @@
           <t>虚构演示主数据，非真实名录判定</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -570,13 +563,6 @@
           <t>虚构演示主数据，非真实名录判定</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -604,13 +590,6 @@
           <t>虚构演示主数据，非真实名录判定</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -618,10 +597,6 @@
           <t>warehouses</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>GW_MAIN</t>
@@ -630,11 +605,6 @@
       <c r="G5" t="n">
         <v>600</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -642,10 +612,6 @@
           <t>warehouses</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>GW_AUX</t>
@@ -654,11 +620,6 @@
       <c r="G6" t="n">
         <v>500</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -666,10 +627,6 @@
           <t>warehouses</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>HW</t>
@@ -678,11 +635,6 @@
       <c r="G7" t="n">
         <v>1000</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -695,11 +647,6 @@
           <t>D-GW</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>G0</t>
@@ -710,9 +657,6 @@
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -725,11 +669,6 @@
           <t>D-OIL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>O0</t>
@@ -740,9 +679,6 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -755,11 +691,6 @@
           <t>D-GW</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>G08</t>
@@ -770,9 +701,6 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -785,11 +713,6 @@
           <t>D-GW</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>G09</t>
@@ -800,9 +723,6 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -815,11 +735,6 @@
           <t>D-OIL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>O08</t>
@@ -830,9 +745,6 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -845,11 +757,6 @@
           <t>D-OIL</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>O09</t>
@@ -860,9 +767,6 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -875,11 +779,6 @@
           <t>D-RAG</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>R08</t>
@@ -890,9 +789,6 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -905,11 +801,6 @@
           <t>D-RAG</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>R09</t>
@@ -920,9 +811,6 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -930,14 +818,6 @@
           <t>production</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -958,14 +838,6 @@
           <t>production</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>2026-09</t>
@@ -1116,11 +988,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1163,11 +1030,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1208,11 +1070,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1253,11 +1110,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1300,11 +1152,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1345,11 +1192,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1390,11 +1232,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1437,11 +1274,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1482,11 +1314,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1527,11 +1354,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1574,11 +1396,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1619,11 +1436,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1664,11 +1476,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1711,11 +1518,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1756,11 +1558,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1801,11 +1598,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1848,11 +1640,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1893,11 +1680,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1938,11 +1720,6 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1978,7 +1755,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>G08</t>
@@ -1989,9 +1765,6 @@
           <t>GW_MAIN</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2027,7 +1800,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>G09</t>
@@ -2038,9 +1810,6 @@
           <t>GW_MAIN</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2076,7 +1845,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>O08</t>
@@ -2087,9 +1855,6 @@
           <t>HW</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2125,7 +1890,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>O09</t>
@@ -2136,9 +1900,6 @@
           <t>HW</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2174,7 +1935,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>R08</t>
@@ -2185,9 +1945,6 @@
           <t>HW</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2223,7 +1980,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>R09</t>
@@ -2234,9 +1990,6 @@
           <t>HW</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2272,7 +2025,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>G0</t>
@@ -2288,8 +2040,6 @@
           <t>G08</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2325,7 +2075,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>G08</t>
@@ -2341,8 +2090,6 @@
           <t>G08</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2378,7 +2125,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>G08</t>
@@ -2394,8 +2140,6 @@
           <t>G09</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2431,7 +2175,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>G09</t>
@@ -2447,8 +2190,6 @@
           <t>G09</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2484,7 +2225,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>O0</t>
@@ -2500,8 +2240,6 @@
           <t>O08</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2537,7 +2275,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>O08</t>
@@ -2553,8 +2290,6 @@
           <t>O08</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2590,7 +2325,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>O08</t>
@@ -2606,8 +2340,6 @@
           <t>O09</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2643,7 +2375,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>O09</t>
@@ -2659,8 +2390,6 @@
           <t>O09</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2696,7 +2425,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>R08</t>
@@ -2712,8 +2440,6 @@
           <t>R08</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2749,7 +2475,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>R09</t>
@@ -2765,8 +2490,6 @@
           <t>R09</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2802,7 +2525,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>G09</t>
@@ -2813,13 +2535,11 @@
           <t>GW_MAIN</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>GW_AUX</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2855,7 +2575,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>G09</t>
@@ -2866,8 +2585,6 @@
           <t>GW_MAIN</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>+</t>
@@ -2908,7 +2625,6 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>R08</t>
@@ -2919,8 +2635,6 @@
           <t>HW</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>-</t>
@@ -3585,7 +3299,6 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4497,7 +4210,6 @@
       <c r="F21" t="n">
         <v>30</v>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>2026-09-29</t>
@@ -4633,7 +4345,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>模拟资料/合同/C-G.txt</t>
+          <t>资料/模拟资料/合同/C-G.txt</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -4686,7 +4398,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>模拟资料/合同/C-O.txt</t>
+          <t>资料/模拟资料/合同/C-O.txt</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -4739,7 +4451,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>模拟资料/合同/C-R.txt</t>
+          <t>资料/模拟资料/合同/C-R.txt</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -5050,7 +4762,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>模拟资料/附件/G08-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/G08-WEIGH.txt</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -5077,7 +4789,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>模拟资料/附件/G08-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/G08-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5104,7 +4816,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>模拟资料/附件/G08-HANDOVER.txt</t>
+          <t>资料/模拟资料/附件/G08-HANDOVER.txt</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5131,7 +4843,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>模拟资料/附件/G09-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/G09-WEIGH.txt</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5158,7 +4870,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>模拟资料/附件/G09-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/G09-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5185,7 +4897,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O08-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/O08-WEIGH.txt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5212,7 +4924,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O08-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/O08-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5239,7 +4951,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O08-MANIFEST.txt</t>
+          <t>资料/模拟资料/附件/O08-MANIFEST.txt</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5266,7 +4978,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O09-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/O09-WEIGH.txt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5293,7 +5005,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O09-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/O09-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5320,7 +5032,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>模拟资料/附件/O09-MANIFEST.txt</t>
+          <t>资料/模拟资料/附件/O09-MANIFEST.txt</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5347,7 +5059,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R08-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/R08-WEIGH.txt</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5374,7 +5086,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R08-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/R08-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5401,7 +5113,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R08-MANIFEST.txt</t>
+          <t>资料/模拟资料/附件/R08-MANIFEST.txt</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5428,7 +5140,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R09-WEIGH.txt</t>
+          <t>资料/模拟资料/附件/R09-WEIGH.txt</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5455,7 +5167,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R09-RECEIVE.txt</t>
+          <t>资料/模拟资料/附件/R09-RECEIVE.txt</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5482,7 +5194,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>模拟资料/附件/R09-MANIFEST.txt</t>
+          <t>资料/模拟资料/附件/R09-MANIFEST.txt</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">

</xml_diff>